<commit_message>
modification page inscription car erreur présente
</commit_message>
<xml_diff>
--- a/CAHIER_DE_TESTS.xlsx
+++ b/CAHIER_DE_TESTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sofian\Desktop\Dev\BackSchool\planity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00754000-F5F3-4BFC-86DC-334F862A516A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB3F98E-22C0-48BD-BC9C-E9248150B362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9AB8989E-98A5-438C-9628-C59E450F55FF}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AB8989E-98A5-438C-9628-C59E450F55FF}"/>
   </bookViews>
   <sheets>
     <sheet name="CAHIER_DE_TESTS" sheetId="1" r:id="rId1"/>
@@ -117,9 +117,6 @@
     <t>Inscription avec email valide</t>
   </si>
   <si>
-    <t>1. Aller sur /register 2. Remplir nom, prÃ©nom, email, mot de passe 3. Cocher CGU 4. Cliquer CrÃ©er mon compte</t>
-  </si>
-  <si>
     <t>Compte crÃ©Ã©, redirection vers /login ou /profile</t>
   </si>
   <si>
@@ -129,9 +126,6 @@
     <t>Inscription sans accepter CGU</t>
   </si>
   <si>
-    <t>1. Aller sur /register 2. Remplir tous les champs 3. Ne pas cocher CGU 4. Cliquer CrÃ©er mon compte</t>
-  </si>
-  <si>
     <t>Message d'erreur, inscription bloquÃ©e</t>
   </si>
   <si>
@@ -153,9 +147,6 @@
     <t>Inscription avec mot de passe faible</t>
   </si>
   <si>
-    <t>1. Aller sur /register 2. Entrer un mot de passe &lt; 8 caractÃ¨res</t>
-  </si>
-  <si>
     <t>Message d'erreur sur le mot de passe</t>
   </si>
   <si>
@@ -1804,6 +1795,15 @@
   </si>
   <si>
     <t>~120 créneaux</t>
+  </si>
+  <si>
+    <t>1. Aller sur /register 2. Remplir nom, prénom, email, mot de passe 3. Cocher CGU 4. Cliquer Créer mon compte</t>
+  </si>
+  <si>
+    <t>1. Aller sur /register 2. Remplir tous les champs 3. Ne pas cocher CGU 4. Cliquer Créer mon compte</t>
+  </si>
+  <si>
+    <t>1. Aller sur /register 2. Entrer un mot de passe &lt; 8 caractères</t>
   </si>
 </sst>
 </file>
@@ -2792,6 +2792,7 @@
     <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="101.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="58.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -2856,7 +2857,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2874,7 +2875,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="B19">
         <v>35</v>
@@ -2882,7 +2883,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B20">
         <v>57</v>
@@ -2890,7 +2891,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B21" s="4">
         <f>B19/B18</f>
@@ -2936,10 +2937,10 @@
         <v>26</v>
       </c>
       <c r="D27" t="s">
+        <v>587</v>
+      </c>
+      <c r="E27" t="s">
         <v>27</v>
-      </c>
-      <c r="E27" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -2947,16 +2948,16 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" t="s">
         <v>29</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
+        <v>588</v>
+      </c>
+      <c r="E28" t="s">
         <v>30</v>
-      </c>
-      <c r="D28" t="s">
-        <v>31</v>
-      </c>
-      <c r="E28" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -2964,16 +2965,16 @@
         <v>24</v>
       </c>
       <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" t="s">
+        <v>32</v>
+      </c>
+      <c r="D29" t="s">
         <v>33</v>
       </c>
-      <c r="C29" t="s">
+      <c r="E29" t="s">
         <v>34</v>
-      </c>
-      <c r="D29" t="s">
-        <v>35</v>
-      </c>
-      <c r="E29" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -2981,16 +2982,16 @@
         <v>24</v>
       </c>
       <c r="B30" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" t="s">
+        <v>589</v>
+      </c>
+      <c r="E30" t="s">
         <v>37</v>
-      </c>
-      <c r="C30" t="s">
-        <v>38</v>
-      </c>
-      <c r="D30" t="s">
-        <v>39</v>
-      </c>
-      <c r="E30" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -2998,1929 +2999,1929 @@
         <v>24</v>
       </c>
       <c r="B31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E31" t="s">
         <v>41</v>
-      </c>
-      <c r="C31" t="s">
-        <v>42</v>
-      </c>
-      <c r="D31" t="s">
-        <v>43</v>
-      </c>
-      <c r="E31" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
         <v>45</v>
       </c>
-      <c r="B32" t="s">
+      <c r="E32" t="s">
         <v>46</v>
-      </c>
-      <c r="C32" t="s">
-        <v>47</v>
-      </c>
-      <c r="D32" t="s">
-        <v>48</v>
-      </c>
-      <c r="E32" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="D33" t="s">
+        <v>49</v>
+      </c>
+      <c r="E33" t="s">
         <v>50</v>
-      </c>
-      <c r="C33" t="s">
-        <v>51</v>
-      </c>
-      <c r="D33" t="s">
-        <v>52</v>
-      </c>
-      <c r="E33" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B34" t="s">
+        <v>51</v>
+      </c>
+      <c r="C34" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E34" t="s">
         <v>54</v>
-      </c>
-      <c r="C34" t="s">
-        <v>55</v>
-      </c>
-      <c r="D34" t="s">
-        <v>56</v>
-      </c>
-      <c r="E34" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" t="s">
+        <v>56</v>
+      </c>
+      <c r="C35" t="s">
+        <v>57</v>
+      </c>
+      <c r="D35" t="s">
         <v>58</v>
       </c>
-      <c r="B35" t="s">
+      <c r="E35" t="s">
         <v>59</v>
-      </c>
-      <c r="C35" t="s">
-        <v>60</v>
-      </c>
-      <c r="D35" t="s">
-        <v>61</v>
-      </c>
-      <c r="E35" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" t="s">
+        <v>62</v>
+      </c>
+      <c r="D36" t="s">
         <v>63</v>
       </c>
-      <c r="B36" t="s">
+      <c r="E36" t="s">
         <v>64</v>
-      </c>
-      <c r="C36" t="s">
-        <v>65</v>
-      </c>
-      <c r="D36" t="s">
-        <v>66</v>
-      </c>
-      <c r="E36" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" t="s">
+        <v>67</v>
+      </c>
+      <c r="E37" t="s">
         <v>68</v>
-      </c>
-      <c r="C37" t="s">
-        <v>69</v>
-      </c>
-      <c r="D37" t="s">
-        <v>70</v>
-      </c>
-      <c r="E37" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B38" t="s">
+        <v>69</v>
+      </c>
+      <c r="C38" t="s">
+        <v>70</v>
+      </c>
+      <c r="D38" t="s">
+        <v>71</v>
+      </c>
+      <c r="E38" t="s">
         <v>72</v>
-      </c>
-      <c r="C38" t="s">
-        <v>73</v>
-      </c>
-      <c r="D38" t="s">
-        <v>74</v>
-      </c>
-      <c r="E38" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>74</v>
+      </c>
+      <c r="B41" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" t="s">
+        <v>76</v>
+      </c>
+      <c r="D41" t="s">
         <v>77</v>
       </c>
-      <c r="B41" t="s">
+      <c r="E41" t="s">
         <v>78</v>
-      </c>
-      <c r="C41" t="s">
-        <v>79</v>
-      </c>
-      <c r="D41" t="s">
-        <v>80</v>
-      </c>
-      <c r="E41" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B42" t="s">
+        <v>79</v>
+      </c>
+      <c r="C42" t="s">
+        <v>80</v>
+      </c>
+      <c r="D42" t="s">
+        <v>81</v>
+      </c>
+      <c r="E42" t="s">
         <v>82</v>
-      </c>
-      <c r="C42" t="s">
-        <v>83</v>
-      </c>
-      <c r="D42" t="s">
-        <v>84</v>
-      </c>
-      <c r="E42" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B43" t="s">
+        <v>83</v>
+      </c>
+      <c r="C43" t="s">
+        <v>84</v>
+      </c>
+      <c r="D43" t="s">
+        <v>85</v>
+      </c>
+      <c r="E43" t="s">
         <v>86</v>
-      </c>
-      <c r="C43" t="s">
-        <v>87</v>
-      </c>
-      <c r="D43" t="s">
-        <v>88</v>
-      </c>
-      <c r="E43" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B44" t="s">
+        <v>87</v>
+      </c>
+      <c r="C44" t="s">
+        <v>88</v>
+      </c>
+      <c r="D44" t="s">
+        <v>89</v>
+      </c>
+      <c r="E44" t="s">
         <v>90</v>
-      </c>
-      <c r="C44" t="s">
-        <v>91</v>
-      </c>
-      <c r="D44" t="s">
-        <v>92</v>
-      </c>
-      <c r="E44" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B45" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" t="s">
+        <v>92</v>
+      </c>
+      <c r="D45" t="s">
+        <v>93</v>
+      </c>
+      <c r="E45" t="s">
         <v>94</v>
-      </c>
-      <c r="C45" t="s">
-        <v>95</v>
-      </c>
-      <c r="D45" t="s">
-        <v>96</v>
-      </c>
-      <c r="E45" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B46" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" t="s">
+        <v>97</v>
+      </c>
+      <c r="E46" t="s">
         <v>98</v>
-      </c>
-      <c r="C46" t="s">
-        <v>99</v>
-      </c>
-      <c r="D46" t="s">
-        <v>100</v>
-      </c>
-      <c r="E46" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B47" t="s">
+        <v>99</v>
+      </c>
+      <c r="C47" t="s">
+        <v>100</v>
+      </c>
+      <c r="D47" t="s">
+        <v>101</v>
+      </c>
+      <c r="E47" t="s">
         <v>102</v>
-      </c>
-      <c r="C47" t="s">
-        <v>103</v>
-      </c>
-      <c r="D47" t="s">
-        <v>104</v>
-      </c>
-      <c r="E47" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>104</v>
+      </c>
+      <c r="B50" t="s">
+        <v>105</v>
+      </c>
+      <c r="C50" t="s">
+        <v>106</v>
+      </c>
+      <c r="D50" t="s">
         <v>107</v>
       </c>
-      <c r="B50" t="s">
+      <c r="E50" t="s">
         <v>108</v>
-      </c>
-      <c r="C50" t="s">
-        <v>109</v>
-      </c>
-      <c r="D50" t="s">
-        <v>110</v>
-      </c>
-      <c r="E50" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B51" t="s">
+        <v>109</v>
+      </c>
+      <c r="C51" t="s">
+        <v>110</v>
+      </c>
+      <c r="D51" t="s">
+        <v>111</v>
+      </c>
+      <c r="E51" t="s">
         <v>112</v>
-      </c>
-      <c r="C51" t="s">
-        <v>113</v>
-      </c>
-      <c r="D51" t="s">
-        <v>114</v>
-      </c>
-      <c r="E51" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B52" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C52" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D52" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E52" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B53" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C53" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D53" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E53" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B54" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C54" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D54" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E54" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B55" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C55" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D55" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E55" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B56" t="s">
+        <v>125</v>
+      </c>
+      <c r="C56" t="s">
+        <v>126</v>
+      </c>
+      <c r="D56" t="s">
+        <v>127</v>
+      </c>
+      <c r="E56" t="s">
         <v>128</v>
-      </c>
-      <c r="C56" t="s">
-        <v>129</v>
-      </c>
-      <c r="D56" t="s">
-        <v>130</v>
-      </c>
-      <c r="E56" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B57" t="s">
+        <v>129</v>
+      </c>
+      <c r="C57" t="s">
+        <v>130</v>
+      </c>
+      <c r="D57" t="s">
+        <v>131</v>
+      </c>
+      <c r="E57" t="s">
         <v>132</v>
-      </c>
-      <c r="C57" t="s">
-        <v>133</v>
-      </c>
-      <c r="D57" t="s">
-        <v>134</v>
-      </c>
-      <c r="E57" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B58" t="s">
+        <v>133</v>
+      </c>
+      <c r="C58" t="s">
+        <v>134</v>
+      </c>
+      <c r="D58" t="s">
+        <v>135</v>
+      </c>
+      <c r="E58" t="s">
         <v>136</v>
-      </c>
-      <c r="C58" t="s">
-        <v>137</v>
-      </c>
-      <c r="D58" t="s">
-        <v>138</v>
-      </c>
-      <c r="E58" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B59" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C59" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D59" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E59" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>141</v>
+      </c>
+      <c r="B62" t="s">
+        <v>142</v>
+      </c>
+      <c r="C62" t="s">
+        <v>143</v>
+      </c>
+      <c r="D62" t="s">
         <v>144</v>
       </c>
-      <c r="B62" t="s">
+      <c r="E62" t="s">
         <v>145</v>
-      </c>
-      <c r="C62" t="s">
-        <v>146</v>
-      </c>
-      <c r="D62" t="s">
-        <v>147</v>
-      </c>
-      <c r="E62" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B63" t="s">
+        <v>146</v>
+      </c>
+      <c r="C63" t="s">
+        <v>147</v>
+      </c>
+      <c r="D63" t="s">
+        <v>148</v>
+      </c>
+      <c r="E63" t="s">
         <v>149</v>
-      </c>
-      <c r="C63" t="s">
-        <v>150</v>
-      </c>
-      <c r="D63" t="s">
-        <v>151</v>
-      </c>
-      <c r="E63" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B64" t="s">
+        <v>150</v>
+      </c>
+      <c r="C64" t="s">
+        <v>151</v>
+      </c>
+      <c r="D64" t="s">
+        <v>152</v>
+      </c>
+      <c r="E64" t="s">
         <v>153</v>
-      </c>
-      <c r="C64" t="s">
-        <v>154</v>
-      </c>
-      <c r="D64" t="s">
-        <v>155</v>
-      </c>
-      <c r="E64" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B65" t="s">
+        <v>154</v>
+      </c>
+      <c r="C65" t="s">
+        <v>155</v>
+      </c>
+      <c r="D65" t="s">
+        <v>156</v>
+      </c>
+      <c r="E65" t="s">
         <v>157</v>
-      </c>
-      <c r="C65" t="s">
-        <v>158</v>
-      </c>
-      <c r="D65" t="s">
-        <v>159</v>
-      </c>
-      <c r="E65" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B66" t="s">
+        <v>158</v>
+      </c>
+      <c r="C66" t="s">
+        <v>159</v>
+      </c>
+      <c r="D66" t="s">
+        <v>160</v>
+      </c>
+      <c r="E66" t="s">
         <v>161</v>
-      </c>
-      <c r="C66" t="s">
-        <v>162</v>
-      </c>
-      <c r="D66" t="s">
-        <v>163</v>
-      </c>
-      <c r="E66" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B67" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C67" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D67" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E67" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B68" t="s">
+        <v>165</v>
+      </c>
+      <c r="C68" t="s">
+        <v>166</v>
+      </c>
+      <c r="D68" t="s">
+        <v>167</v>
+      </c>
+      <c r="E68" t="s">
         <v>168</v>
-      </c>
-      <c r="C68" t="s">
-        <v>169</v>
-      </c>
-      <c r="D68" t="s">
-        <v>170</v>
-      </c>
-      <c r="E68" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B69" t="s">
+        <v>169</v>
+      </c>
+      <c r="C69" t="s">
+        <v>170</v>
+      </c>
+      <c r="D69" t="s">
+        <v>171</v>
+      </c>
+      <c r="E69" t="s">
         <v>172</v>
-      </c>
-      <c r="C69" t="s">
-        <v>173</v>
-      </c>
-      <c r="D69" t="s">
-        <v>174</v>
-      </c>
-      <c r="E69" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B70" t="s">
+        <v>173</v>
+      </c>
+      <c r="C70" t="s">
+        <v>174</v>
+      </c>
+      <c r="D70" t="s">
+        <v>175</v>
+      </c>
+      <c r="E70" t="s">
         <v>176</v>
-      </c>
-      <c r="C70" t="s">
-        <v>177</v>
-      </c>
-      <c r="D70" t="s">
-        <v>178</v>
-      </c>
-      <c r="E70" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B71" t="s">
+        <v>177</v>
+      </c>
+      <c r="C71" t="s">
+        <v>178</v>
+      </c>
+      <c r="D71" t="s">
+        <v>179</v>
+      </c>
+      <c r="E71" t="s">
         <v>180</v>
-      </c>
-      <c r="C71" t="s">
-        <v>181</v>
-      </c>
-      <c r="D71" t="s">
-        <v>182</v>
-      </c>
-      <c r="E71" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C72" t="s">
+        <v>182</v>
+      </c>
+      <c r="D72" t="s">
+        <v>183</v>
+      </c>
+      <c r="E72" t="s">
         <v>184</v>
-      </c>
-      <c r="C72" t="s">
-        <v>185</v>
-      </c>
-      <c r="D72" t="s">
-        <v>186</v>
-      </c>
-      <c r="E72" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>186</v>
+      </c>
+      <c r="B75" t="s">
+        <v>187</v>
+      </c>
+      <c r="C75" t="s">
+        <v>188</v>
+      </c>
+      <c r="D75" t="s">
         <v>189</v>
       </c>
-      <c r="B75" t="s">
+      <c r="E75" t="s">
         <v>190</v>
-      </c>
-      <c r="C75" t="s">
-        <v>191</v>
-      </c>
-      <c r="D75" t="s">
-        <v>192</v>
-      </c>
-      <c r="E75" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B76" t="s">
+        <v>191</v>
+      </c>
+      <c r="C76" t="s">
+        <v>192</v>
+      </c>
+      <c r="D76" t="s">
+        <v>193</v>
+      </c>
+      <c r="E76" t="s">
         <v>194</v>
-      </c>
-      <c r="C76" t="s">
-        <v>195</v>
-      </c>
-      <c r="D76" t="s">
-        <v>196</v>
-      </c>
-      <c r="E76" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B77" t="s">
+        <v>195</v>
+      </c>
+      <c r="C77" t="s">
+        <v>196</v>
+      </c>
+      <c r="D77" t="s">
+        <v>197</v>
+      </c>
+      <c r="E77" t="s">
         <v>198</v>
-      </c>
-      <c r="C77" t="s">
-        <v>199</v>
-      </c>
-      <c r="D77" t="s">
-        <v>200</v>
-      </c>
-      <c r="E77" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B78" t="s">
+        <v>199</v>
+      </c>
+      <c r="C78" t="s">
+        <v>200</v>
+      </c>
+      <c r="D78" t="s">
+        <v>201</v>
+      </c>
+      <c r="E78" t="s">
         <v>202</v>
-      </c>
-      <c r="C78" t="s">
-        <v>203</v>
-      </c>
-      <c r="D78" t="s">
-        <v>204</v>
-      </c>
-      <c r="E78" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B79" t="s">
+        <v>203</v>
+      </c>
+      <c r="C79" t="s">
+        <v>204</v>
+      </c>
+      <c r="D79" t="s">
+        <v>205</v>
+      </c>
+      <c r="E79" t="s">
         <v>206</v>
-      </c>
-      <c r="C79" t="s">
-        <v>207</v>
-      </c>
-      <c r="D79" t="s">
-        <v>208</v>
-      </c>
-      <c r="E79" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B80" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C80" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D80" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E80" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B81" t="s">
+        <v>210</v>
+      </c>
+      <c r="C81" t="s">
+        <v>211</v>
+      </c>
+      <c r="D81" t="s">
+        <v>212</v>
+      </c>
+      <c r="E81" t="s">
         <v>213</v>
-      </c>
-      <c r="C81" t="s">
-        <v>214</v>
-      </c>
-      <c r="D81" t="s">
-        <v>215</v>
-      </c>
-      <c r="E81" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>215</v>
+      </c>
+      <c r="B84" t="s">
+        <v>216</v>
+      </c>
+      <c r="C84" t="s">
+        <v>217</v>
+      </c>
+      <c r="D84" t="s">
         <v>218</v>
       </c>
-      <c r="B84" t="s">
+      <c r="E84" t="s">
         <v>219</v>
-      </c>
-      <c r="C84" t="s">
-        <v>220</v>
-      </c>
-      <c r="D84" t="s">
-        <v>221</v>
-      </c>
-      <c r="E84" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B85" t="s">
+        <v>220</v>
+      </c>
+      <c r="C85" t="s">
+        <v>221</v>
+      </c>
+      <c r="D85" t="s">
+        <v>222</v>
+      </c>
+      <c r="E85" t="s">
         <v>223</v>
-      </c>
-      <c r="C85" t="s">
-        <v>224</v>
-      </c>
-      <c r="D85" t="s">
-        <v>225</v>
-      </c>
-      <c r="E85" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B86" t="s">
+        <v>224</v>
+      </c>
+      <c r="C86" t="s">
+        <v>225</v>
+      </c>
+      <c r="D86" t="s">
+        <v>226</v>
+      </c>
+      <c r="E86" t="s">
         <v>227</v>
-      </c>
-      <c r="C86" t="s">
-        <v>228</v>
-      </c>
-      <c r="D86" t="s">
-        <v>229</v>
-      </c>
-      <c r="E86" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B87" t="s">
+        <v>228</v>
+      </c>
+      <c r="C87" t="s">
+        <v>229</v>
+      </c>
+      <c r="D87" t="s">
+        <v>230</v>
+      </c>
+      <c r="E87" t="s">
         <v>231</v>
-      </c>
-      <c r="C87" t="s">
-        <v>232</v>
-      </c>
-      <c r="D87" t="s">
-        <v>233</v>
-      </c>
-      <c r="E87" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B88" t="s">
+        <v>232</v>
+      </c>
+      <c r="C88" t="s">
+        <v>233</v>
+      </c>
+      <c r="D88" t="s">
+        <v>234</v>
+      </c>
+      <c r="E88" t="s">
         <v>235</v>
-      </c>
-      <c r="C88" t="s">
-        <v>236</v>
-      </c>
-      <c r="D88" t="s">
-        <v>237</v>
-      </c>
-      <c r="E88" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B89" t="s">
+        <v>236</v>
+      </c>
+      <c r="C89" t="s">
+        <v>237</v>
+      </c>
+      <c r="D89" t="s">
+        <v>238</v>
+      </c>
+      <c r="E89" t="s">
         <v>239</v>
-      </c>
-      <c r="C89" t="s">
-        <v>240</v>
-      </c>
-      <c r="D89" t="s">
-        <v>241</v>
-      </c>
-      <c r="E89" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B90" t="s">
+        <v>240</v>
+      </c>
+      <c r="C90" t="s">
+        <v>241</v>
+      </c>
+      <c r="D90" t="s">
+        <v>242</v>
+      </c>
+      <c r="E90" t="s">
         <v>243</v>
-      </c>
-      <c r="C90" t="s">
-        <v>244</v>
-      </c>
-      <c r="D90" t="s">
-        <v>245</v>
-      </c>
-      <c r="E90" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B91" t="s">
+        <v>244</v>
+      </c>
+      <c r="C91" t="s">
+        <v>245</v>
+      </c>
+      <c r="D91" t="s">
+        <v>246</v>
+      </c>
+      <c r="E91" t="s">
         <v>247</v>
-      </c>
-      <c r="C91" t="s">
-        <v>248</v>
-      </c>
-      <c r="D91" t="s">
-        <v>249</v>
-      </c>
-      <c r="E91" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>249</v>
+      </c>
+      <c r="B94" t="s">
+        <v>250</v>
+      </c>
+      <c r="C94" t="s">
+        <v>251</v>
+      </c>
+      <c r="D94" t="s">
         <v>252</v>
       </c>
-      <c r="B94" t="s">
+      <c r="E94" t="s">
         <v>253</v>
-      </c>
-      <c r="C94" t="s">
-        <v>254</v>
-      </c>
-      <c r="D94" t="s">
-        <v>255</v>
-      </c>
-      <c r="E94" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B95" t="s">
+        <v>254</v>
+      </c>
+      <c r="C95" t="s">
+        <v>255</v>
+      </c>
+      <c r="D95" t="s">
+        <v>256</v>
+      </c>
+      <c r="E95" t="s">
         <v>257</v>
-      </c>
-      <c r="C95" t="s">
-        <v>258</v>
-      </c>
-      <c r="D95" t="s">
-        <v>259</v>
-      </c>
-      <c r="E95" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B96" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C96" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D96" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E96" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B97" t="s">
+        <v>261</v>
+      </c>
+      <c r="C97" t="s">
+        <v>262</v>
+      </c>
+      <c r="D97" t="s">
+        <v>263</v>
+      </c>
+      <c r="E97" t="s">
         <v>264</v>
-      </c>
-      <c r="C97" t="s">
-        <v>265</v>
-      </c>
-      <c r="D97" t="s">
-        <v>266</v>
-      </c>
-      <c r="E97" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B98" t="s">
+        <v>265</v>
+      </c>
+      <c r="C98" t="s">
+        <v>266</v>
+      </c>
+      <c r="D98" t="s">
+        <v>267</v>
+      </c>
+      <c r="E98" t="s">
         <v>268</v>
-      </c>
-      <c r="C98" t="s">
-        <v>269</v>
-      </c>
-      <c r="D98" t="s">
-        <v>270</v>
-      </c>
-      <c r="E98" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B99" t="s">
+        <v>269</v>
+      </c>
+      <c r="C99" t="s">
+        <v>270</v>
+      </c>
+      <c r="D99" t="s">
+        <v>271</v>
+      </c>
+      <c r="E99" t="s">
         <v>272</v>
-      </c>
-      <c r="C99" t="s">
-        <v>273</v>
-      </c>
-      <c r="D99" t="s">
-        <v>274</v>
-      </c>
-      <c r="E99" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B100" t="s">
+        <v>273</v>
+      </c>
+      <c r="C100" t="s">
+        <v>274</v>
+      </c>
+      <c r="D100" t="s">
+        <v>275</v>
+      </c>
+      <c r="E100" t="s">
         <v>276</v>
-      </c>
-      <c r="C100" t="s">
-        <v>277</v>
-      </c>
-      <c r="D100" t="s">
-        <v>278</v>
-      </c>
-      <c r="E100" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B101" t="s">
+        <v>277</v>
+      </c>
+      <c r="C101" t="s">
+        <v>278</v>
+      </c>
+      <c r="D101" t="s">
+        <v>279</v>
+      </c>
+      <c r="E101" t="s">
         <v>280</v>
-      </c>
-      <c r="C101" t="s">
-        <v>281</v>
-      </c>
-      <c r="D101" t="s">
-        <v>282</v>
-      </c>
-      <c r="E101" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B102" t="s">
+        <v>281</v>
+      </c>
+      <c r="C102" t="s">
+        <v>282</v>
+      </c>
+      <c r="D102" t="s">
+        <v>283</v>
+      </c>
+      <c r="E102" t="s">
         <v>284</v>
-      </c>
-      <c r="C102" t="s">
-        <v>285</v>
-      </c>
-      <c r="D102" t="s">
-        <v>286</v>
-      </c>
-      <c r="E102" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B103" t="s">
+        <v>285</v>
+      </c>
+      <c r="C103" t="s">
+        <v>286</v>
+      </c>
+      <c r="D103" t="s">
+        <v>287</v>
+      </c>
+      <c r="E103" t="s">
         <v>288</v>
-      </c>
-      <c r="C103" t="s">
-        <v>289</v>
-      </c>
-      <c r="D103" t="s">
-        <v>290</v>
-      </c>
-      <c r="E103" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B104" t="s">
+        <v>289</v>
+      </c>
+      <c r="C104" t="s">
+        <v>290</v>
+      </c>
+      <c r="D104" t="s">
+        <v>291</v>
+      </c>
+      <c r="E104" t="s">
         <v>292</v>
-      </c>
-      <c r="C104" t="s">
-        <v>293</v>
-      </c>
-      <c r="D104" t="s">
-        <v>294</v>
-      </c>
-      <c r="E104" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B105" t="s">
+        <v>293</v>
+      </c>
+      <c r="C105" t="s">
+        <v>294</v>
+      </c>
+      <c r="D105" t="s">
+        <v>295</v>
+      </c>
+      <c r="E105" t="s">
         <v>296</v>
-      </c>
-      <c r="C105" t="s">
-        <v>297</v>
-      </c>
-      <c r="D105" t="s">
-        <v>298</v>
-      </c>
-      <c r="E105" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B106" t="s">
+        <v>297</v>
+      </c>
+      <c r="C106" t="s">
+        <v>298</v>
+      </c>
+      <c r="D106" t="s">
+        <v>299</v>
+      </c>
+      <c r="E106" t="s">
         <v>300</v>
-      </c>
-      <c r="C106" t="s">
-        <v>301</v>
-      </c>
-      <c r="D106" t="s">
-        <v>302</v>
-      </c>
-      <c r="E106" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B107" t="s">
+        <v>301</v>
+      </c>
+      <c r="C107" t="s">
+        <v>302</v>
+      </c>
+      <c r="D107" t="s">
+        <v>303</v>
+      </c>
+      <c r="E107" t="s">
         <v>304</v>
-      </c>
-      <c r="C107" t="s">
-        <v>305</v>
-      </c>
-      <c r="D107" t="s">
-        <v>306</v>
-      </c>
-      <c r="E107" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B108" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C108" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D108" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="E108" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>309</v>
+      </c>
+      <c r="B111" t="s">
+        <v>310</v>
+      </c>
+      <c r="C111" t="s">
+        <v>311</v>
+      </c>
+      <c r="D111" t="s">
         <v>312</v>
       </c>
-      <c r="B111" t="s">
+      <c r="E111" t="s">
         <v>313</v>
-      </c>
-      <c r="C111" t="s">
-        <v>314</v>
-      </c>
-      <c r="D111" t="s">
-        <v>315</v>
-      </c>
-      <c r="E111" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B112" t="s">
+        <v>314</v>
+      </c>
+      <c r="C112" t="s">
+        <v>315</v>
+      </c>
+      <c r="D112" t="s">
+        <v>316</v>
+      </c>
+      <c r="E112" t="s">
         <v>317</v>
-      </c>
-      <c r="C112" t="s">
-        <v>318</v>
-      </c>
-      <c r="D112" t="s">
-        <v>319</v>
-      </c>
-      <c r="E112" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B113" t="s">
+        <v>318</v>
+      </c>
+      <c r="C113" t="s">
+        <v>319</v>
+      </c>
+      <c r="D113" t="s">
+        <v>320</v>
+      </c>
+      <c r="E113" t="s">
         <v>321</v>
-      </c>
-      <c r="C113" t="s">
-        <v>322</v>
-      </c>
-      <c r="D113" t="s">
-        <v>323</v>
-      </c>
-      <c r="E113" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B114" t="s">
+        <v>322</v>
+      </c>
+      <c r="C114" t="s">
+        <v>323</v>
+      </c>
+      <c r="D114" t="s">
+        <v>324</v>
+      </c>
+      <c r="E114" t="s">
         <v>325</v>
-      </c>
-      <c r="C114" t="s">
-        <v>326</v>
-      </c>
-      <c r="D114" t="s">
-        <v>327</v>
-      </c>
-      <c r="E114" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B115" t="s">
+        <v>326</v>
+      </c>
+      <c r="C115" t="s">
+        <v>327</v>
+      </c>
+      <c r="D115" t="s">
+        <v>328</v>
+      </c>
+      <c r="E115" t="s">
         <v>329</v>
-      </c>
-      <c r="C115" t="s">
-        <v>330</v>
-      </c>
-      <c r="D115" t="s">
-        <v>331</v>
-      </c>
-      <c r="E115" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B116" t="s">
+        <v>330</v>
+      </c>
+      <c r="C116" t="s">
+        <v>331</v>
+      </c>
+      <c r="D116" t="s">
+        <v>332</v>
+      </c>
+      <c r="E116" t="s">
         <v>333</v>
-      </c>
-      <c r="C116" t="s">
-        <v>334</v>
-      </c>
-      <c r="D116" t="s">
-        <v>335</v>
-      </c>
-      <c r="E116" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
+        <v>335</v>
+      </c>
+      <c r="B119" t="s">
+        <v>336</v>
+      </c>
+      <c r="C119" t="s">
+        <v>337</v>
+      </c>
+      <c r="D119" t="s">
         <v>338</v>
       </c>
-      <c r="B119" t="s">
+      <c r="E119" t="s">
         <v>339</v>
-      </c>
-      <c r="C119" t="s">
-        <v>340</v>
-      </c>
-      <c r="D119" t="s">
-        <v>341</v>
-      </c>
-      <c r="E119" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B120" t="s">
+        <v>340</v>
+      </c>
+      <c r="C120" t="s">
+        <v>341</v>
+      </c>
+      <c r="D120" t="s">
+        <v>342</v>
+      </c>
+      <c r="E120" t="s">
         <v>343</v>
-      </c>
-      <c r="C120" t="s">
-        <v>344</v>
-      </c>
-      <c r="D120" t="s">
-        <v>345</v>
-      </c>
-      <c r="E120" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B121" t="s">
+        <v>344</v>
+      </c>
+      <c r="C121" t="s">
+        <v>345</v>
+      </c>
+      <c r="D121" t="s">
+        <v>346</v>
+      </c>
+      <c r="E121" t="s">
         <v>347</v>
-      </c>
-      <c r="C121" t="s">
-        <v>348</v>
-      </c>
-      <c r="D121" t="s">
-        <v>349</v>
-      </c>
-      <c r="E121" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B122" t="s">
+        <v>348</v>
+      </c>
+      <c r="C122" t="s">
+        <v>349</v>
+      </c>
+      <c r="D122" t="s">
+        <v>350</v>
+      </c>
+      <c r="E122" t="s">
         <v>351</v>
-      </c>
-      <c r="C122" t="s">
-        <v>352</v>
-      </c>
-      <c r="D122" t="s">
-        <v>353</v>
-      </c>
-      <c r="E122" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B123" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C123" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="D123" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E123" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B124" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C124" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="D124" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E124" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B125" t="s">
+        <v>357</v>
+      </c>
+      <c r="C125" t="s">
+        <v>358</v>
+      </c>
+      <c r="D125" t="s">
+        <v>359</v>
+      </c>
+      <c r="E125" t="s">
         <v>360</v>
-      </c>
-      <c r="C125" t="s">
-        <v>361</v>
-      </c>
-      <c r="D125" t="s">
-        <v>362</v>
-      </c>
-      <c r="E125" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B126" t="s">
+        <v>361</v>
+      </c>
+      <c r="C126" t="s">
+        <v>362</v>
+      </c>
+      <c r="D126" t="s">
+        <v>363</v>
+      </c>
+      <c r="E126" t="s">
         <v>364</v>
-      </c>
-      <c r="C126" t="s">
-        <v>365</v>
-      </c>
-      <c r="D126" t="s">
-        <v>366</v>
-      </c>
-      <c r="E126" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
+        <v>366</v>
+      </c>
+      <c r="B129" t="s">
+        <v>367</v>
+      </c>
+      <c r="C129" t="s">
+        <v>368</v>
+      </c>
+      <c r="D129" t="s">
         <v>369</v>
       </c>
-      <c r="B129" t="s">
+      <c r="E129" t="s">
         <v>370</v>
-      </c>
-      <c r="C129" t="s">
-        <v>371</v>
-      </c>
-      <c r="D129" t="s">
-        <v>372</v>
-      </c>
-      <c r="E129" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B130" t="s">
+        <v>371</v>
+      </c>
+      <c r="C130" t="s">
+        <v>372</v>
+      </c>
+      <c r="D130" t="s">
+        <v>373</v>
+      </c>
+      <c r="E130" t="s">
         <v>374</v>
-      </c>
-      <c r="C130" t="s">
-        <v>375</v>
-      </c>
-      <c r="D130" t="s">
-        <v>376</v>
-      </c>
-      <c r="E130" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B131" t="s">
+        <v>375</v>
+      </c>
+      <c r="C131" t="s">
+        <v>376</v>
+      </c>
+      <c r="D131" t="s">
+        <v>377</v>
+      </c>
+      <c r="E131" t="s">
         <v>378</v>
-      </c>
-      <c r="C131" t="s">
-        <v>379</v>
-      </c>
-      <c r="D131" t="s">
-        <v>380</v>
-      </c>
-      <c r="E131" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B132" t="s">
+        <v>379</v>
+      </c>
+      <c r="C132" t="s">
+        <v>380</v>
+      </c>
+      <c r="D132" t="s">
+        <v>381</v>
+      </c>
+      <c r="E132" t="s">
         <v>382</v>
-      </c>
-      <c r="C132" t="s">
-        <v>383</v>
-      </c>
-      <c r="D132" t="s">
-        <v>384</v>
-      </c>
-      <c r="E132" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B133" t="s">
+        <v>383</v>
+      </c>
+      <c r="C133" t="s">
+        <v>384</v>
+      </c>
+      <c r="D133" t="s">
+        <v>385</v>
+      </c>
+      <c r="E133" t="s">
         <v>386</v>
-      </c>
-      <c r="C133" t="s">
-        <v>387</v>
-      </c>
-      <c r="D133" t="s">
-        <v>388</v>
-      </c>
-      <c r="E133" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B134" t="s">
+        <v>387</v>
+      </c>
+      <c r="C134" t="s">
+        <v>388</v>
+      </c>
+      <c r="D134" t="s">
+        <v>389</v>
+      </c>
+      <c r="E134" t="s">
         <v>390</v>
-      </c>
-      <c r="C134" t="s">
-        <v>391</v>
-      </c>
-      <c r="D134" t="s">
-        <v>392</v>
-      </c>
-      <c r="E134" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B135" t="s">
+        <v>391</v>
+      </c>
+      <c r="C135" t="s">
+        <v>392</v>
+      </c>
+      <c r="D135" t="s">
+        <v>393</v>
+      </c>
+      <c r="E135" t="s">
         <v>394</v>
-      </c>
-      <c r="C135" t="s">
-        <v>395</v>
-      </c>
-      <c r="D135" t="s">
-        <v>396</v>
-      </c>
-      <c r="E135" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B136" t="s">
+        <v>395</v>
+      </c>
+      <c r="C136" t="s">
+        <v>396</v>
+      </c>
+      <c r="D136" t="s">
+        <v>397</v>
+      </c>
+      <c r="E136" t="s">
         <v>398</v>
-      </c>
-      <c r="C136" t="s">
-        <v>399</v>
-      </c>
-      <c r="D136" t="s">
-        <v>400</v>
-      </c>
-      <c r="E136" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B137" t="s">
+        <v>399</v>
+      </c>
+      <c r="C137" t="s">
+        <v>400</v>
+      </c>
+      <c r="D137" t="s">
+        <v>401</v>
+      </c>
+      <c r="E137" t="s">
         <v>402</v>
-      </c>
-      <c r="C137" t="s">
-        <v>403</v>
-      </c>
-      <c r="D137" t="s">
-        <v>404</v>
-      </c>
-      <c r="E137" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B138" t="s">
+        <v>403</v>
+      </c>
+      <c r="C138" t="s">
+        <v>404</v>
+      </c>
+      <c r="D138" t="s">
+        <v>405</v>
+      </c>
+      <c r="E138" t="s">
         <v>406</v>
-      </c>
-      <c r="C138" t="s">
-        <v>407</v>
-      </c>
-      <c r="D138" t="s">
-        <v>408</v>
-      </c>
-      <c r="E138" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B139" t="s">
+        <v>407</v>
+      </c>
+      <c r="C139" t="s">
+        <v>408</v>
+      </c>
+      <c r="D139" t="s">
+        <v>409</v>
+      </c>
+      <c r="E139" t="s">
         <v>410</v>
-      </c>
-      <c r="C139" t="s">
-        <v>411</v>
-      </c>
-      <c r="D139" t="s">
-        <v>412</v>
-      </c>
-      <c r="E139" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
+        <v>412</v>
+      </c>
+      <c r="B142" t="s">
+        <v>413</v>
+      </c>
+      <c r="C142" t="s">
+        <v>414</v>
+      </c>
+      <c r="D142" t="s">
         <v>415</v>
       </c>
-      <c r="B142" t="s">
+      <c r="E142" t="s">
         <v>416</v>
-      </c>
-      <c r="C142" t="s">
-        <v>417</v>
-      </c>
-      <c r="D142" t="s">
-        <v>418</v>
-      </c>
-      <c r="E142" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B143" t="s">
+        <v>417</v>
+      </c>
+      <c r="C143" t="s">
+        <v>418</v>
+      </c>
+      <c r="D143" t="s">
+        <v>419</v>
+      </c>
+      <c r="E143" t="s">
         <v>420</v>
-      </c>
-      <c r="C143" t="s">
-        <v>421</v>
-      </c>
-      <c r="D143" t="s">
-        <v>422</v>
-      </c>
-      <c r="E143" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B144" t="s">
+        <v>421</v>
+      </c>
+      <c r="C144" t="s">
+        <v>422</v>
+      </c>
+      <c r="D144" t="s">
+        <v>423</v>
+      </c>
+      <c r="E144" t="s">
         <v>424</v>
-      </c>
-      <c r="C144" t="s">
-        <v>425</v>
-      </c>
-      <c r="D144" t="s">
-        <v>426</v>
-      </c>
-      <c r="E144" t="s">
-        <v>427</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B145" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="C145" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="D145" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="E145" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B146" t="s">
+        <v>428</v>
+      </c>
+      <c r="C146" t="s">
+        <v>429</v>
+      </c>
+      <c r="D146" t="s">
+        <v>430</v>
+      </c>
+      <c r="E146" t="s">
         <v>431</v>
-      </c>
-      <c r="C146" t="s">
-        <v>432</v>
-      </c>
-      <c r="D146" t="s">
-        <v>433</v>
-      </c>
-      <c r="E146" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B147" t="s">
+        <v>432</v>
+      </c>
+      <c r="C147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D147" t="s">
+        <v>434</v>
+      </c>
+      <c r="E147" t="s">
         <v>435</v>
-      </c>
-      <c r="C147" t="s">
-        <v>436</v>
-      </c>
-      <c r="D147" t="s">
-        <v>437</v>
-      </c>
-      <c r="E147" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B148" t="s">
+        <v>436</v>
+      </c>
+      <c r="C148" t="s">
+        <v>437</v>
+      </c>
+      <c r="D148" t="s">
+        <v>438</v>
+      </c>
+      <c r="E148" t="s">
         <v>439</v>
-      </c>
-      <c r="C148" t="s">
-        <v>440</v>
-      </c>
-      <c r="D148" t="s">
-        <v>441</v>
-      </c>
-      <c r="E148" t="s">
-        <v>442</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B149" t="s">
+        <v>440</v>
+      </c>
+      <c r="C149" t="s">
+        <v>441</v>
+      </c>
+      <c r="D149" t="s">
+        <v>442</v>
+      </c>
+      <c r="E149" t="s">
         <v>443</v>
-      </c>
-      <c r="C149" t="s">
-        <v>444</v>
-      </c>
-      <c r="D149" t="s">
-        <v>445</v>
-      </c>
-      <c r="E149" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B150" t="s">
+        <v>444</v>
+      </c>
+      <c r="C150" t="s">
+        <v>445</v>
+      </c>
+      <c r="D150" t="s">
+        <v>446</v>
+      </c>
+      <c r="E150" t="s">
         <v>447</v>
-      </c>
-      <c r="C150" t="s">
-        <v>448</v>
-      </c>
-      <c r="D150" t="s">
-        <v>449</v>
-      </c>
-      <c r="E150" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B151" t="s">
+        <v>448</v>
+      </c>
+      <c r="C151" t="s">
+        <v>449</v>
+      </c>
+      <c r="D151" t="s">
+        <v>450</v>
+      </c>
+      <c r="E151" t="s">
         <v>451</v>
-      </c>
-      <c r="C151" t="s">
-        <v>452</v>
-      </c>
-      <c r="D151" t="s">
-        <v>453</v>
-      </c>
-      <c r="E151" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B152" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="C152" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D152" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E152" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
+        <v>456</v>
+      </c>
+      <c r="B155" t="s">
+        <v>457</v>
+      </c>
+      <c r="C155" t="s">
+        <v>458</v>
+      </c>
+      <c r="D155" t="s">
         <v>459</v>
       </c>
-      <c r="B155" t="s">
-        <v>460</v>
-      </c>
-      <c r="C155" t="s">
-        <v>461</v>
-      </c>
-      <c r="D155" t="s">
-        <v>462</v>
-      </c>
       <c r="E155" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B156" t="s">
+        <v>460</v>
+      </c>
+      <c r="C156" t="s">
+        <v>461</v>
+      </c>
+      <c r="D156" t="s">
+        <v>462</v>
+      </c>
+      <c r="E156" t="s">
         <v>463</v>
-      </c>
-      <c r="C156" t="s">
-        <v>464</v>
-      </c>
-      <c r="D156" t="s">
-        <v>465</v>
-      </c>
-      <c r="E156" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B157" t="s">
+        <v>464</v>
+      </c>
+      <c r="C157" t="s">
+        <v>465</v>
+      </c>
+      <c r="D157" t="s">
+        <v>466</v>
+      </c>
+      <c r="E157" t="s">
         <v>467</v>
-      </c>
-      <c r="C157" t="s">
-        <v>468</v>
-      </c>
-      <c r="D157" t="s">
-        <v>469</v>
-      </c>
-      <c r="E157" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B158" t="s">
+        <v>468</v>
+      </c>
+      <c r="C158" t="s">
+        <v>469</v>
+      </c>
+      <c r="D158" t="s">
+        <v>470</v>
+      </c>
+      <c r="E158" t="s">
         <v>471</v>
-      </c>
-      <c r="C158" t="s">
-        <v>472</v>
-      </c>
-      <c r="D158" t="s">
-        <v>473</v>
-      </c>
-      <c r="E158" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B159" t="s">
+        <v>472</v>
+      </c>
+      <c r="C159" t="s">
+        <v>473</v>
+      </c>
+      <c r="D159" t="s">
+        <v>474</v>
+      </c>
+      <c r="E159" t="s">
         <v>475</v>
-      </c>
-      <c r="C159" t="s">
-        <v>476</v>
-      </c>
-      <c r="D159" t="s">
-        <v>477</v>
-      </c>
-      <c r="E159" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
+        <v>477</v>
+      </c>
+      <c r="B162" t="s">
+        <v>478</v>
+      </c>
+      <c r="C162" t="s">
+        <v>479</v>
+      </c>
+      <c r="D162" t="s">
         <v>480</v>
       </c>
-      <c r="B162" t="s">
+      <c r="E162" t="s">
         <v>481</v>
-      </c>
-      <c r="C162" t="s">
-        <v>482</v>
-      </c>
-      <c r="D162" t="s">
-        <v>483</v>
-      </c>
-      <c r="E162" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="B163" t="s">
+        <v>482</v>
+      </c>
+      <c r="C163" t="s">
+        <v>483</v>
+      </c>
+      <c r="D163" t="s">
+        <v>484</v>
+      </c>
+      <c r="E163" t="s">
         <v>485</v>
-      </c>
-      <c r="C163" t="s">
-        <v>486</v>
-      </c>
-      <c r="D163" t="s">
-        <v>487</v>
-      </c>
-      <c r="E163" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="B164" t="s">
+        <v>486</v>
+      </c>
+      <c r="C164" t="s">
+        <v>487</v>
+      </c>
+      <c r="D164" t="s">
+        <v>488</v>
+      </c>
+      <c r="E164" t="s">
         <v>489</v>
-      </c>
-      <c r="C164" t="s">
-        <v>490</v>
-      </c>
-      <c r="D164" t="s">
-        <v>491</v>
-      </c>
-      <c r="E164" t="s">
-        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -4950,348 +4951,348 @@
   <sheetData>
     <row r="2" spans="2:16" ht="42" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="3" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
     </row>
     <row r="5" spans="2:16" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>498</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>501</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>504</v>
-      </c>
       <c r="G5" s="9" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="P5" s="9" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F6" s="8" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="P6" s="9" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
     </row>
     <row r="7" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F7" s="8" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
     </row>
     <row r="8" spans="2:16" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F8" s="8" t="s">
+        <v>507</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>508</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>538</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>539</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>559</v>
+      </c>
+      <c r="O8" s="9" t="s">
+        <v>560</v>
+      </c>
+      <c r="P8" s="9" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F9" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="J9" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>541</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>562</v>
+      </c>
+      <c r="O9" s="9" t="s">
+        <v>563</v>
+      </c>
+      <c r="P9" s="9" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F10" s="8" t="s">
         <v>511</v>
       </c>
-      <c r="J8" s="8" t="s">
-        <v>541</v>
-      </c>
-      <c r="K8" s="9" t="s">
+      <c r="G10" s="9" t="s">
+        <v>512</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>542</v>
       </c>
-      <c r="N8" s="8" t="s">
-        <v>562</v>
-      </c>
-      <c r="O8" s="9" t="s">
-        <v>563</v>
-      </c>
-      <c r="P8" s="9" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="9" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F9" s="8" t="s">
-        <v>512</v>
-      </c>
-      <c r="G9" s="9" t="s">
+      <c r="K10" s="9" t="s">
+        <v>543</v>
+      </c>
+      <c r="N10" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="O10" s="9" t="s">
+        <v>566</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F11" s="8" t="s">
         <v>513</v>
       </c>
-      <c r="J9" s="8" t="s">
-        <v>543</v>
-      </c>
-      <c r="K9" s="9" t="s">
+      <c r="G11" s="9" t="s">
+        <v>514</v>
+      </c>
+      <c r="J11" s="8" t="s">
         <v>544</v>
       </c>
-      <c r="N9" s="8" t="s">
-        <v>565</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>566</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="10" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F10" s="8" t="s">
-        <v>514</v>
-      </c>
-      <c r="G10" s="9" t="s">
+      <c r="K11" s="9" t="s">
+        <v>545</v>
+      </c>
+      <c r="N11" s="8" t="s">
+        <v>568</v>
+      </c>
+      <c r="O11" s="9" t="s">
+        <v>569</v>
+      </c>
+      <c r="P11" s="9" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F12" s="8" t="s">
         <v>515</v>
       </c>
-      <c r="J10" s="8" t="s">
-        <v>545</v>
-      </c>
-      <c r="K10" s="9" t="s">
+      <c r="G12" s="9" t="s">
+        <v>516</v>
+      </c>
+      <c r="J12" s="8" t="s">
         <v>546</v>
       </c>
-      <c r="N10" s="8" t="s">
-        <v>568</v>
-      </c>
-      <c r="O10" s="9" t="s">
-        <v>569</v>
-      </c>
-      <c r="P10" s="9" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="11" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F11" s="8" t="s">
-        <v>516</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>517</v>
-      </c>
-      <c r="J11" s="8" t="s">
+      <c r="K12" s="9" t="s">
         <v>547</v>
       </c>
-      <c r="K11" s="9" t="s">
-        <v>548</v>
-      </c>
-      <c r="N11" s="8" t="s">
+      <c r="N12" s="8" t="s">
         <v>571</v>
       </c>
-      <c r="O11" s="9" t="s">
+      <c r="O12" s="9" t="s">
         <v>572</v>
       </c>
-      <c r="P11" s="9" t="s">
+      <c r="P12" s="9" t="s">
         <v>573</v>
-      </c>
-    </row>
-    <row r="12" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="8" t="s">
-        <v>518</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>519</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>549</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>550</v>
-      </c>
-      <c r="N12" s="8" t="s">
-        <v>574</v>
-      </c>
-      <c r="O12" s="9" t="s">
-        <v>575</v>
-      </c>
-      <c r="P12" s="9" t="s">
-        <v>576</v>
       </c>
     </row>
     <row r="13" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F13" s="8" t="s">
+        <v>517</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>518</v>
+      </c>
+      <c r="N13" s="9" t="s">
+        <v>574</v>
+      </c>
+      <c r="O13" s="9" t="s">
+        <v>574</v>
+      </c>
+      <c r="P13" s="9" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F14" s="8" t="s">
+        <v>519</v>
+      </c>
+      <c r="G14" s="9" t="s">
         <v>520</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>521</v>
-      </c>
-      <c r="N13" s="9" t="s">
+      <c r="N14" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="O14" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="P14" s="9" t="s">
         <v>577</v>
-      </c>
-      <c r="O13" s="9" t="s">
-        <v>577</v>
-      </c>
-      <c r="P13" s="9" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="14" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="8" t="s">
-        <v>522</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>523</v>
-      </c>
-      <c r="N14" s="8" t="s">
-        <v>578</v>
-      </c>
-      <c r="O14" s="9" t="s">
-        <v>579</v>
-      </c>
-      <c r="P14" s="9" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="15" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F15" s="8" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
     </row>
     <row r="16" spans="2:16" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F16" s="8" t="s">
+        <v>523</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F17" s="8" t="s">
+        <v>525</v>
+      </c>
+      <c r="G17" s="9" t="s">
         <v>526</v>
       </c>
-      <c r="G16" s="9" t="s">
+    </row>
+    <row r="18" spans="6:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="8" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="17" spans="6:7" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F17" s="8" t="s">
+      <c r="G18" s="9" t="s">
         <v>528</v>
       </c>
-      <c r="G17" s="9" t="s">
+    </row>
+    <row r="19" spans="6:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F19" s="8" t="s">
         <v>529</v>
       </c>
-    </row>
-    <row r="18" spans="6:7" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F18" s="8" t="s">
+      <c r="G19" s="9" t="s">
         <v>530</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="19" spans="6:7" ht="41.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F19" s="8" t="s">
-        <v>532</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="53" spans="2:3" ht="26.25" x14ac:dyDescent="0.25">
       <c r="B53" s="10" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
     </row>
     <row r="54" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B55" s="5" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
     </row>
     <row r="56" spans="2:3" ht="100.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
     </row>
     <row r="57" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="9" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
     </row>
     <row r="58" spans="2:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B58" s="9" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
     </row>
   </sheetData>

</xml_diff>